<commit_message>
Top Tier: redact EIN from NetProfit workbook A3 (all five sheets)
A3 now reads "Top Tier Roofing & Remodeling, LLC   |   prepared 31 August 2026".
Regenerated from work/scripts/build_netprofit_xlsx_260831.py; cell-by-cell diff
against the pre-change archive shows exactly five differences, all A3.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXWU5qwaBEzjQR7ueAqAJv
</commit_message>
<xml_diff>
--- a/toptier/files/TopTier.NetProfit.2025v2026.260831.xlsx
+++ b/toptier/files/TopTier.NetProfit.2025v2026.260831.xlsx
@@ -656,7 +656,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Top Tier Roofing &amp; Remodeling, LLC   |   EIN 99-3048348   |   prepared 31 August 2026</t>
+          <t>Top Tier Roofing &amp; Remodeling, LLC   |   prepared 31 August 2026</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Top Tier Roofing &amp; Remodeling, LLC   |   EIN 99-3048348   |   prepared 31 August 2026</t>
+          <t>Top Tier Roofing &amp; Remodeling, LLC   |   prepared 31 August 2026</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Top Tier Roofing &amp; Remodeling, LLC   |   EIN 99-3048348   |   prepared 31 August 2026</t>
+          <t>Top Tier Roofing &amp; Remodeling, LLC   |   prepared 31 August 2026</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Top Tier Roofing &amp; Remodeling, LLC   |   EIN 99-3048348   |   prepared 31 August 2026</t>
+          <t>Top Tier Roofing &amp; Remodeling, LLC   |   prepared 31 August 2026</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Top Tier Roofing &amp; Remodeling, LLC   |   EIN 99-3048348   |   prepared 31 August 2026</t>
+          <t>Top Tier Roofing &amp; Remodeling, LLC   |   prepared 31 August 2026</t>
         </is>
       </c>
     </row>

</xml_diff>